<commit_message>
vault backup: 2026-08-10 09:48:54
</commit_message>
<xml_diff>
--- a/ContabilidadeFinanceira/Aulas/08.10/TreinoDFs.xlsx
+++ b/ContabilidadeFinanceira/Aulas/08.10/TreinoDFs.xlsx
@@ -14,7 +14,8 @@
     <sheet name="C_Caso1" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="C_Caso2" sheetId="5" state="visible" r:id="rId7"/>
     <sheet name="D_Pegadinhas" sheetId="6" state="visible" r:id="rId8"/>
-    <sheet name="Gabarito" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="E_Transacoes" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="Gabarito" sheetId="8" state="visible" r:id="rId10"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="369" uniqueCount="221">
   <si>
     <t xml:space="preserve">Treino: DFs principais (ContabilidadeFinanceira, 10.08.2026)</t>
   </si>
@@ -49,7 +50,10 @@
     <t xml:space="preserve">5. Não abre a aba Gabarito antes de terminar. A correção automática já te diz se acertou.</t>
   </si>
   <si>
-    <t xml:space="preserve">Ordem sugerida (tempo total ~40 min): A conceitos, B classificação, C caso 1, C caso 2, D pegadinhas.</t>
+    <t xml:space="preserve">Ordem sugerida (tempo total ~50 min): A conceitos, B classificação, C caso 1, C caso 2, D pegadinhas, E transações.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O Bloco E treina o formato exato da planilha da videoaula (tema 3, aula de hoje): registrar transações e ver a equação fechar coluna a coluna.</t>
   </si>
   <si>
     <t xml:space="preserve">Exemplo de como funciona: a primeira linha da aba B_Classificacao já vem respondida como demonstração.</t>
@@ -385,6 +389,99 @@
     <t xml:space="preserve">Empresa comprou máquina de 200 à vista em dezembro. Efeito imediato no lucro do ano? No caixa? Nos lucros dos próximos anos?</t>
   </si>
   <si>
+    <t xml:space="preserve">Bloco E: registro de transações, formato da planilha da videoaula (tema 3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T1. Sócios integralizam capital de 50.000 em dinheiro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T2. Compra de equipamento à vista por 30.000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T3. Compra de mercadorias por 12.000, metade à vista, metade a prazo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T4. Venda de mercadorias por 9.000 à vista; o custo era 6.000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T5. Venda de mercadorias por 8.000 a prazo; o custo era 4.000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T6. Pagamento de 4.000 das contas a pagar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Preenche o efeito de cada transação em cada conta (positivo ou negativo). Saldo final e checks são automáticos.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Conta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Saldo final</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Caixa   [ativo]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contas a Receber   [ativo]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estoque   [ativo]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Imobilizado   [ativo]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contas a Pagar   [passivo/PL]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Capital Social   [passivo/PL]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lucros Acumulados   [passivo/PL]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diferença da equação por transação (tem que dar 0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Agora o filme do período (DRE e DFC, valores em cima das mesmas transações):</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Receita de vendas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(=) Lucro do período</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FCO (recebeu de cliente menos pagou fornecedor)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FCI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FCF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A variação do caixa bateu com o saldo final da conta Caixa? Lucro 7.000 com FCO negativo: quem explica a diferença?</t>
+  </si>
+  <si>
     <t xml:space="preserve">Gabarito</t>
   </si>
   <si>
@@ -400,12 +497,18 @@
     <t xml:space="preserve">Bloco A</t>
   </si>
   <si>
+    <t xml:space="preserve">Bloco E: deltas por transação (fechados na mão a partir do enunciado da aba E)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Bloco B (mesma linha da aba B_Classificacao)</t>
   </si>
   <si>
     <t xml:space="preserve">C_Caso1: Receita líquida</t>
   </si>
   <si>
+    <t xml:space="preserve">Caixa</t>
+  </si>
+  <si>
     <t xml:space="preserve">C_Caso1: (-) CMV</t>
   </si>
   <si>
@@ -415,6 +518,9 @@
     <t xml:space="preserve">A1. RA: o que aconteceu e pra onde vamos, na voz da gestão. BP: onde o dinheiro está aplicado e de onde veio. DRE: resultado das operações do período. DFC: principais entradas e saídas de caixa.</t>
   </si>
   <si>
+    <t xml:space="preserve">Contas a Receber</t>
+  </si>
+  <si>
     <t xml:space="preserve">C_Caso1: (=) Lucro bruto</t>
   </si>
   <si>
@@ -424,6 +530,9 @@
     <t xml:space="preserve">A2. BP é foto de uma data; DRE e DFC são filmes de um período. Posição vs desempenho: comparar duas fotos do BP exige os filmes pra explicar o que mudou.</t>
   </si>
   <si>
+    <t xml:space="preserve">Estoque</t>
+  </si>
+  <si>
     <t xml:space="preserve">C_Caso1: (-) Despesas de vendas</t>
   </si>
   <si>
@@ -433,6 +542,9 @@
     <t xml:space="preserve">A3. Os dois lados são a mesma coisa vista de ângulos diferentes: esquerdo mostra onde o dinheiro está aplicado, direito mostra de onde veio (terceiros ou sócios). Todo recurso aplicado tem origem; se não bate, tem erro.</t>
   </si>
   <si>
+    <t xml:space="preserve">Imobilizado</t>
+  </si>
+  <si>
     <t xml:space="preserve">DRE</t>
   </si>
   <si>
@@ -445,6 +557,9 @@
     <t xml:space="preserve">A4. Por função responde 'pra que gastei': lucro bruto isola o valor agregado da atividade-fim, EBIT isola a operação inteira, LL isola o que sobra pro acionista depois de banco e governo. Por natureza responderia 'com que gastei' e misturaria as camadas.</t>
   </si>
   <si>
+    <t xml:space="preserve">Contas a Pagar</t>
+  </si>
+  <si>
     <t xml:space="preserve">DFC</t>
   </si>
   <si>
@@ -457,18 +572,27 @@
     <t xml:space="preserve">A5. DRE é competência, caixa é sobrevivência. Varejista que vende a prazo longo e estoca agressivo mostra lucro alto com FCO fraco; sem caixa pra pagar fornecedor, quebra com DRE bonita.</t>
   </si>
   <si>
+    <t xml:space="preserve">Capital Social</t>
+  </si>
+  <si>
     <t xml:space="preserve">C_Caso1: (+/-) Resultado financeiro</t>
   </si>
   <si>
     <t xml:space="preserve">A6. Baixo: é a gestão escrevendo sobre si mesma, sem o rigor de auditoria das DFs. Serve de contexto e guia de leitura; toda afirmação se confere contra os números.</t>
   </si>
   <si>
+    <t xml:space="preserve">Lucros Acumulados</t>
+  </si>
+  <si>
     <t xml:space="preserve">C_Caso1: (=) LAIR</t>
   </si>
   <si>
     <t xml:space="preserve">A7. Consolidado é o grupo econômico (visão econômica); controladora é a pessoa jurídica sozinha (visão jurídica). Holding 'Participações' sozinha não opera nada.</t>
   </si>
   <si>
+    <t xml:space="preserve">Bloco E: DRE e DFC do período</t>
+  </si>
+  <si>
     <t xml:space="preserve">RA</t>
   </si>
   <si>
@@ -505,6 +629,12 @@
     <t xml:space="preserve">C_Caso1: (+) Aumento de fornecedores</t>
   </si>
   <si>
+    <t xml:space="preserve">Bloco E: resposta discursiva</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sim, 19.000 nos dois. O lucro é competência (vendas de 17.000, custo 10.000); o FCO é caixa: só recebeu 9.000 (a venda a prazo ainda não entrou) e pagou 10.000. A diferença estacionou em contas a receber (+8.000) e no giro de estoque/fornecedores.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Despesa administrativa</t>
   </si>
   <si>
@@ -535,9 +665,6 @@
     <t xml:space="preserve">C_Caso1: Δ Imobilizado (capex menos D&amp;A)</t>
   </si>
   <si>
-    <t xml:space="preserve">FCI</t>
-  </si>
-  <si>
     <t xml:space="preserve">C_Caso1: (=) Δ Ativo total</t>
   </si>
   <si>
@@ -545,9 +672,6 @@
   </si>
   <si>
     <t xml:space="preserve">C_Caso1: Δ Fornecedores</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FCF</t>
   </si>
   <si>
     <t xml:space="preserve">C_Caso1: Δ Empréstimos</t>
@@ -726,7 +850,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="29">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -813,6 +937,22 @@
     </xf>
     <xf numFmtId="164" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
@@ -1099,7 +1239,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B2:B12"/>
+  <dimension ref="B2:B13"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="100"/>
@@ -1143,7 +1283,7 @@
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="3"/>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="3" t="s">
         <v>7</v>
       </c>
@@ -1151,6 +1291,11 @@
     <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="3" t="s">
         <v>8</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B13" s="3" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -1178,15 +1323,15 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1194,7 +1339,7 @@
         <v>1</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C4" s="8"/>
     </row>
@@ -1203,7 +1348,7 @@
         <v>2</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C5" s="8"/>
     </row>
@@ -1212,7 +1357,7 @@
         <v>3</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C6" s="8"/>
     </row>
@@ -1221,7 +1366,7 @@
         <v>4</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C7" s="8"/>
     </row>
@@ -1230,7 +1375,7 @@
         <v>5</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C8" s="8"/>
     </row>
@@ -1239,7 +1384,7 @@
         <v>6</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C9" s="8"/>
     </row>
@@ -1248,7 +1393,7 @@
         <v>7</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C10" s="8"/>
     </row>
@@ -1279,37 +1424,37 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="9" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D5" s="12" t="str">
         <f aca="false">IF(C5="","",IF(C5=Gabarito!C5,"✔","✗"))</f>
@@ -1321,7 +1466,7 @@
         <v>1</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C6" s="13"/>
       <c r="D6" s="12" t="str">
@@ -1334,7 +1479,7 @@
         <v>2</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C7" s="13"/>
       <c r="D7" s="12" t="str">
@@ -1347,7 +1492,7 @@
         <v>3</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C8" s="13"/>
       <c r="D8" s="12" t="str">
@@ -1360,7 +1505,7 @@
         <v>4</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C9" s="13"/>
       <c r="D9" s="12" t="str">
@@ -1373,7 +1518,7 @@
         <v>5</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C10" s="13"/>
       <c r="D10" s="12" t="str">
@@ -1386,7 +1531,7 @@
         <v>6</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C11" s="13"/>
       <c r="D11" s="12" t="str">
@@ -1399,7 +1544,7 @@
         <v>7</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C12" s="13"/>
       <c r="D12" s="12" t="str">
@@ -1409,7 +1554,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C13" s="9" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D13" s="14" t="str">
         <f aca="false">COUNTIF(D6:D12,"✔")&amp;" / 7"</f>
@@ -1418,21 +1563,21 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="9" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D16" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1440,7 +1585,7 @@
         <v>0</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C17" s="13"/>
       <c r="D17" s="12" t="str">
@@ -1453,7 +1598,7 @@
         <v>1</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C18" s="13"/>
       <c r="D18" s="12" t="str">
@@ -1466,7 +1611,7 @@
         <v>2</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C19" s="13"/>
       <c r="D19" s="12" t="str">
@@ -1479,7 +1624,7 @@
         <v>3</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C20" s="13"/>
       <c r="D20" s="12" t="str">
@@ -1492,7 +1637,7 @@
         <v>4</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C21" s="13"/>
       <c r="D21" s="12" t="str">
@@ -1505,7 +1650,7 @@
         <v>5</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C22" s="13"/>
       <c r="D22" s="12" t="str">
@@ -1518,7 +1663,7 @@
         <v>6</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C23" s="13"/>
       <c r="D23" s="12" t="str">
@@ -1531,7 +1676,7 @@
         <v>7</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C24" s="13"/>
       <c r="D24" s="12" t="str">
@@ -1541,7 +1686,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C25" s="9" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D25" s="14" t="str">
         <f aca="false">COUNTIF(D18:D24,"✔")&amp;" / 7"</f>
@@ -1550,21 +1695,21 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="9" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="10" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D28" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1572,7 +1717,7 @@
         <v>0</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C29" s="13"/>
       <c r="D29" s="12" t="str">
@@ -1585,7 +1730,7 @@
         <v>1</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C30" s="13"/>
       <c r="D30" s="12" t="str">
@@ -1598,7 +1743,7 @@
         <v>2</v>
       </c>
       <c r="B31" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C31" s="13"/>
       <c r="D31" s="12" t="str">
@@ -1611,7 +1756,7 @@
         <v>3</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C32" s="13"/>
       <c r="D32" s="12" t="str">
@@ -1624,7 +1769,7 @@
         <v>4</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C33" s="13"/>
       <c r="D33" s="12" t="str">
@@ -1637,7 +1782,7 @@
         <v>5</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C34" s="13"/>
       <c r="D34" s="12" t="str">
@@ -1650,7 +1795,7 @@
         <v>6</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C35" s="13"/>
       <c r="D35" s="12" t="str">
@@ -1663,7 +1808,7 @@
         <v>7</v>
       </c>
       <c r="B36" s="7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C36" s="13"/>
       <c r="D36" s="12" t="str">
@@ -1673,7 +1818,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C37" s="9" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D37" s="14" t="str">
         <f aca="false">COUNTIF(D30:D36,"✔")&amp;" / 7"</f>
@@ -1729,25 +1874,25 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="5" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="15" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C5" s="16" t="n">
         <v>1000</v>
@@ -1755,7 +1900,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="15" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C6" s="16" t="n">
         <v>600</v>
@@ -1763,7 +1908,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="15" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C7" s="16" t="n">
         <v>120</v>
@@ -1771,7 +1916,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="15" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C8" s="16" t="n">
         <v>80</v>
@@ -1779,7 +1924,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="15" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C9" s="16" t="n">
         <v>30</v>
@@ -1787,7 +1932,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="15" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C10" s="16" t="n">
         <v>40</v>
@@ -1795,7 +1940,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="15" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C11" s="16" t="n">
         <v>10</v>
@@ -1803,7 +1948,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="15" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C12" s="17" t="n">
         <v>0.3</v>
@@ -1811,7 +1956,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="15" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C13" s="16" t="n">
         <v>50</v>
@@ -1819,7 +1964,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="15" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C14" s="16" t="n">
         <v>40</v>
@@ -1827,7 +1972,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="15" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C15" s="16" t="n">
         <v>20</v>
@@ -1835,7 +1980,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="15" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C16" s="16" t="n">
         <v>100</v>
@@ -1843,7 +1988,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="15" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C17" s="16" t="n">
         <v>60</v>
@@ -1851,7 +1996,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="15" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C18" s="16" t="n">
         <v>0</v>
@@ -1859,7 +2004,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="15" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C19" s="16" t="n">
         <v>30</v>
@@ -1867,7 +2012,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="15" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C20" s="16" t="n">
         <v>41</v>
@@ -1875,23 +2020,23 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="9" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D23" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="18" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C24" s="19"/>
       <c r="D24" s="12" t="str">
@@ -1901,7 +2046,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="18" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C25" s="19"/>
       <c r="D25" s="12" t="str">
@@ -1911,7 +2056,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="18" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C26" s="19"/>
       <c r="D26" s="12" t="str">
@@ -1921,7 +2066,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="18" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C27" s="19"/>
       <c r="D27" s="12" t="str">
@@ -1931,7 +2076,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="18" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C28" s="19"/>
       <c r="D28" s="12" t="str">
@@ -1941,7 +2086,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="18" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C29" s="19"/>
       <c r="D29" s="12" t="str">
@@ -1951,7 +2096,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="18" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C30" s="19"/>
       <c r="D30" s="12" t="str">
@@ -1961,7 +2106,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="18" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C31" s="19"/>
       <c r="D31" s="12" t="str">
@@ -1971,7 +2116,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="18" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C32" s="19"/>
       <c r="D32" s="12" t="str">
@@ -1981,7 +2126,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="18" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C33" s="19"/>
       <c r="D33" s="12" t="str">
@@ -1991,23 +2136,23 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="9" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C36" s="10" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D36" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="18" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C37" s="20"/>
       <c r="D37" s="12" t="str">
@@ -2017,23 +2162,23 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="9" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B40" s="5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C40" s="10" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D40" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B41" s="18" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C41" s="19"/>
       <c r="D41" s="12" t="str">
@@ -2043,7 +2188,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="18" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C42" s="19"/>
       <c r="D42" s="12" t="str">
@@ -2053,7 +2198,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B43" s="18" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C43" s="19"/>
       <c r="D43" s="12" t="str">
@@ -2063,7 +2208,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B44" s="18" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C44" s="19"/>
       <c r="D44" s="12" t="str">
@@ -2073,7 +2218,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B45" s="18" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C45" s="19"/>
       <c r="D45" s="12" t="str">
@@ -2083,7 +2228,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B46" s="18" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C46" s="19"/>
       <c r="D46" s="12" t="str">
@@ -2093,23 +2238,23 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B48" s="9" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B49" s="5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C49" s="10" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D49" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B50" s="18" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C50" s="19"/>
       <c r="D50" s="12" t="str">
@@ -2119,7 +2264,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B51" s="18" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C51" s="19"/>
       <c r="D51" s="12" t="str">
@@ -2129,7 +2274,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B52" s="18" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C52" s="19"/>
       <c r="D52" s="12" t="str">
@@ -2139,7 +2284,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B53" s="18" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C53" s="19"/>
       <c r="D53" s="12" t="str">
@@ -2149,7 +2294,7 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B54" s="18" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C54" s="19"/>
       <c r="D54" s="12" t="str">
@@ -2159,23 +2304,23 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B56" s="9" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B57" s="5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C57" s="10" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D57" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B58" s="18" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C58" s="19"/>
       <c r="D58" s="12" t="str">
@@ -2185,7 +2330,7 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B59" s="18" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C59" s="19"/>
       <c r="D59" s="12" t="str">
@@ -2195,7 +2340,7 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B60" s="18" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C60" s="19"/>
       <c r="D60" s="12" t="str">
@@ -2205,7 +2350,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B61" s="18" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C61" s="19"/>
       <c r="D61" s="12" t="str">
@@ -2215,7 +2360,7 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B62" s="18" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C62" s="19"/>
       <c r="D62" s="12" t="str">
@@ -2225,7 +2370,7 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B63" s="18" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C63" s="19"/>
       <c r="D63" s="12" t="str">
@@ -2235,7 +2380,7 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B64" s="18" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C64" s="19"/>
       <c r="D64" s="12" t="str">
@@ -2245,7 +2390,7 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B65" s="18" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C65" s="19"/>
       <c r="D65" s="12" t="str">
@@ -2255,7 +2400,7 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B66" s="18" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C66" s="19"/>
       <c r="D66" s="12" t="str">
@@ -2265,7 +2410,7 @@
     </row>
     <row r="68" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B68" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="54.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2311,25 +2456,25 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="4" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="9" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="5" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="15" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C5" s="16" t="n">
         <v>1200</v>
@@ -2337,7 +2482,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="15" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C6" s="16" t="n">
         <v>660</v>
@@ -2345,7 +2490,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="15" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C7" s="16" t="n">
         <v>150</v>
@@ -2353,7 +2498,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="15" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C8" s="16" t="n">
         <v>90</v>
@@ -2361,7 +2506,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="15" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C9" s="16" t="n">
         <v>40</v>
@@ -2369,7 +2514,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="15" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C10" s="16" t="n">
         <v>60</v>
@@ -2377,7 +2522,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="15" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C11" s="16" t="n">
         <v>20</v>
@@ -2385,7 +2530,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="15" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C12" s="17" t="n">
         <v>0.3</v>
@@ -2393,7 +2538,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="15" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C13" s="16" t="n">
         <v>80</v>
@@ -2401,7 +2546,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="15" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C14" s="16" t="n">
         <v>30</v>
@@ -2409,7 +2554,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="15" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C15" s="16" t="n">
         <v>50</v>
@@ -2417,7 +2562,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="15" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C16" s="16" t="n">
         <v>120</v>
@@ -2425,7 +2570,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="15" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C17" s="16" t="n">
         <v>0</v>
@@ -2433,7 +2578,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="15" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C18" s="16" t="n">
         <v>40</v>
@@ -2441,7 +2586,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="15" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C19" s="16" t="n">
         <v>50</v>
@@ -2449,7 +2594,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="15" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C20" s="16" t="n">
         <v>100</v>
@@ -2457,23 +2602,23 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="9" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D23" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="18" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C24" s="19"/>
       <c r="D24" s="12" t="str">
@@ -2483,7 +2628,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="18" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C25" s="19"/>
       <c r="D25" s="12" t="str">
@@ -2493,7 +2638,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="18" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C26" s="19"/>
       <c r="D26" s="12" t="str">
@@ -2503,7 +2648,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="18" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C27" s="19"/>
       <c r="D27" s="12" t="str">
@@ -2513,7 +2658,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="18" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C28" s="19"/>
       <c r="D28" s="12" t="str">
@@ -2523,7 +2668,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="18" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C29" s="19"/>
       <c r="D29" s="12" t="str">
@@ -2533,7 +2678,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="18" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C30" s="19"/>
       <c r="D30" s="12" t="str">
@@ -2543,7 +2688,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="18" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C31" s="19"/>
       <c r="D31" s="12" t="str">
@@ -2553,7 +2698,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="18" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C32" s="19"/>
       <c r="D32" s="12" t="str">
@@ -2563,7 +2708,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="18" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C33" s="19"/>
       <c r="D33" s="12" t="str">
@@ -2573,23 +2718,23 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="9" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C36" s="10" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D36" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="18" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C37" s="20"/>
       <c r="D37" s="12" t="str">
@@ -2599,23 +2744,23 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="9" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B40" s="5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C40" s="10" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D40" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B41" s="18" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C41" s="19"/>
       <c r="D41" s="12" t="str">
@@ -2625,7 +2770,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="18" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C42" s="19"/>
       <c r="D42" s="12" t="str">
@@ -2635,7 +2780,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B43" s="18" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C43" s="19"/>
       <c r="D43" s="12" t="str">
@@ -2645,7 +2790,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B44" s="18" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C44" s="19"/>
       <c r="D44" s="12" t="str">
@@ -2655,7 +2800,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B45" s="18" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C45" s="19"/>
       <c r="D45" s="12" t="str">
@@ -2665,7 +2810,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B46" s="18" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C46" s="19"/>
       <c r="D46" s="12" t="str">
@@ -2675,23 +2820,23 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B48" s="9" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B49" s="5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C49" s="10" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D49" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B50" s="18" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C50" s="19"/>
       <c r="D50" s="12" t="str">
@@ -2701,7 +2846,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B51" s="18" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C51" s="19"/>
       <c r="D51" s="12" t="str">
@@ -2711,7 +2856,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B52" s="18" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C52" s="19"/>
       <c r="D52" s="12" t="str">
@@ -2721,7 +2866,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B53" s="18" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C53" s="19"/>
       <c r="D53" s="12" t="str">
@@ -2731,7 +2876,7 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B54" s="18" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C54" s="19"/>
       <c r="D54" s="12" t="str">
@@ -2741,23 +2886,23 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B56" s="9" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B57" s="5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C57" s="10" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D57" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B58" s="18" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C58" s="19"/>
       <c r="D58" s="12" t="str">
@@ -2767,7 +2912,7 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B59" s="18" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C59" s="19"/>
       <c r="D59" s="12" t="str">
@@ -2777,7 +2922,7 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B60" s="18" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C60" s="19"/>
       <c r="D60" s="12" t="str">
@@ -2787,7 +2932,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B61" s="18" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C61" s="19"/>
       <c r="D61" s="12" t="str">
@@ -2797,7 +2942,7 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B62" s="18" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C62" s="19"/>
       <c r="D62" s="12" t="str">
@@ -2807,7 +2952,7 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B63" s="18" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C63" s="19"/>
       <c r="D63" s="12" t="str">
@@ -2817,7 +2962,7 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B64" s="18" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C64" s="19"/>
       <c r="D64" s="12" t="str">
@@ -2827,7 +2972,7 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B65" s="18" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C65" s="19"/>
       <c r="D65" s="12" t="str">
@@ -2837,7 +2982,7 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B66" s="18" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C66" s="19"/>
       <c r="D66" s="12" t="str">
@@ -2847,7 +2992,7 @@
     </row>
     <row r="68" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B68" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="54.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2891,15 +3036,15 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="4" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2907,7 +3052,7 @@
         <v>1</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C4" s="8"/>
     </row>
@@ -2916,7 +3061,7 @@
         <v>2</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C5" s="8"/>
     </row>
@@ -2925,7 +3070,7 @@
         <v>3</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C6" s="8"/>
     </row>
@@ -2934,7 +3079,7 @@
         <v>4</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C7" s="8"/>
     </row>
@@ -2943,7 +3088,7 @@
         <v>5</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C8" s="8"/>
     </row>
@@ -2963,7 +3108,372 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B1:H36"/>
+  <dimension ref="A1:I30"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="2" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="4" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="22" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="22" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="22" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="22" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="22" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="22" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="9" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>129</v>
+      </c>
+      <c r="C11" s="10" t="s">
+        <v>130</v>
+      </c>
+      <c r="D11" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="E11" s="10" t="s">
+        <v>132</v>
+      </c>
+      <c r="F11" s="10" t="s">
+        <v>133</v>
+      </c>
+      <c r="G11" s="10" t="s">
+        <v>134</v>
+      </c>
+      <c r="H11" s="10" t="s">
+        <v>135</v>
+      </c>
+      <c r="I11" s="10" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="18" t="s">
+        <v>136</v>
+      </c>
+      <c r="B12" s="19"/>
+      <c r="C12" s="19"/>
+      <c r="D12" s="19"/>
+      <c r="E12" s="19"/>
+      <c r="F12" s="19"/>
+      <c r="G12" s="19"/>
+      <c r="H12" s="23" t="n">
+        <f aca="false">SUM(B12:G12)</f>
+        <v>0</v>
+      </c>
+      <c r="I12" s="12" t="str">
+        <f aca="false">IF(COUNT(B12:G12)=0,"",IF(ABS(H12-Gabarito!$P$3)&lt;0.5,"✔","✗"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="18" t="s">
+        <v>137</v>
+      </c>
+      <c r="B13" s="19"/>
+      <c r="C13" s="19"/>
+      <c r="D13" s="19"/>
+      <c r="E13" s="19"/>
+      <c r="F13" s="19"/>
+      <c r="G13" s="19"/>
+      <c r="H13" s="23" t="n">
+        <f aca="false">SUM(B13:G13)</f>
+        <v>0</v>
+      </c>
+      <c r="I13" s="12" t="str">
+        <f aca="false">IF(COUNT(B13:G13)=0,"",IF(ABS(H13-Gabarito!$P$4)&lt;0.5,"✔","✗"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="18" t="s">
+        <v>138</v>
+      </c>
+      <c r="B14" s="19"/>
+      <c r="C14" s="19"/>
+      <c r="D14" s="19"/>
+      <c r="E14" s="19"/>
+      <c r="F14" s="19"/>
+      <c r="G14" s="19"/>
+      <c r="H14" s="23" t="n">
+        <f aca="false">SUM(B14:G14)</f>
+        <v>0</v>
+      </c>
+      <c r="I14" s="12" t="str">
+        <f aca="false">IF(COUNT(B14:G14)=0,"",IF(ABS(H14-Gabarito!$P$5)&lt;0.5,"✔","✗"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="18" t="s">
+        <v>139</v>
+      </c>
+      <c r="B15" s="19"/>
+      <c r="C15" s="19"/>
+      <c r="D15" s="19"/>
+      <c r="E15" s="19"/>
+      <c r="F15" s="19"/>
+      <c r="G15" s="19"/>
+      <c r="H15" s="23" t="n">
+        <f aca="false">SUM(B15:G15)</f>
+        <v>0</v>
+      </c>
+      <c r="I15" s="12" t="str">
+        <f aca="false">IF(COUNT(B15:G15)=0,"",IF(ABS(H15-Gabarito!$P$6)&lt;0.5,"✔","✗"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="18" t="s">
+        <v>140</v>
+      </c>
+      <c r="B16" s="19"/>
+      <c r="C16" s="19"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="19"/>
+      <c r="F16" s="19"/>
+      <c r="G16" s="19"/>
+      <c r="H16" s="23" t="n">
+        <f aca="false">SUM(B16:G16)</f>
+        <v>0</v>
+      </c>
+      <c r="I16" s="12" t="str">
+        <f aca="false">IF(COUNT(B16:G16)=0,"",IF(ABS(H16-Gabarito!$P$7)&lt;0.5,"✔","✗"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="18" t="s">
+        <v>141</v>
+      </c>
+      <c r="B17" s="19"/>
+      <c r="C17" s="19"/>
+      <c r="D17" s="19"/>
+      <c r="E17" s="19"/>
+      <c r="F17" s="19"/>
+      <c r="G17" s="19"/>
+      <c r="H17" s="23" t="n">
+        <f aca="false">SUM(B17:G17)</f>
+        <v>0</v>
+      </c>
+      <c r="I17" s="12" t="str">
+        <f aca="false">IF(COUNT(B17:G17)=0,"",IF(ABS(H17-Gabarito!$P$8)&lt;0.5,"✔","✗"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="18" t="s">
+        <v>142</v>
+      </c>
+      <c r="B18" s="19"/>
+      <c r="C18" s="19"/>
+      <c r="D18" s="19"/>
+      <c r="E18" s="19"/>
+      <c r="F18" s="19"/>
+      <c r="G18" s="19"/>
+      <c r="H18" s="23" t="n">
+        <f aca="false">SUM(B18:G18)</f>
+        <v>0</v>
+      </c>
+      <c r="I18" s="12" t="str">
+        <f aca="false">IF(COUNT(B18:G18)=0,"",IF(ABS(H18-Gabarito!$P$9)&lt;0.5,"✔","✗"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="24" t="s">
+        <v>143</v>
+      </c>
+      <c r="B19" s="25" t="n">
+        <f aca="false">(B12+B13+B14+B15)-(B16+B17+B18)</f>
+        <v>0</v>
+      </c>
+      <c r="C19" s="25" t="n">
+        <f aca="false">(C12+C13+C14+C15)-(C16+C17+C18)</f>
+        <v>0</v>
+      </c>
+      <c r="D19" s="25" t="n">
+        <f aca="false">(D12+D13+D14+D15)-(D16+D17+D18)</f>
+        <v>0</v>
+      </c>
+      <c r="E19" s="25" t="n">
+        <f aca="false">(E12+E13+E14+E15)-(E16+E17+E18)</f>
+        <v>0</v>
+      </c>
+      <c r="F19" s="25" t="n">
+        <f aca="false">(F12+F13+F14+F15)-(F16+F17+F18)</f>
+        <v>0</v>
+      </c>
+      <c r="G19" s="25" t="n">
+        <f aca="false">(G12+G13+G14+G15)-(G16+G17+G18)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="9" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="18" t="s">
+        <v>145</v>
+      </c>
+      <c r="B22" s="19"/>
+      <c r="C22" s="12" t="str">
+        <f aca="false">IF(B22="","",IF(ABS(B22-Gabarito!$P$11)&lt;0.5,"✔","✗"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="18" t="s">
+        <v>78</v>
+      </c>
+      <c r="B23" s="19"/>
+      <c r="C23" s="12" t="str">
+        <f aca="false">IF(B23="","",IF(ABS(B23-Gabarito!$P$12)&lt;0.5,"✔","✗"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="18" t="s">
+        <v>146</v>
+      </c>
+      <c r="B24" s="19"/>
+      <c r="C24" s="12" t="str">
+        <f aca="false">IF(B24="","",IF(ABS(B24-Gabarito!$P$13)&lt;0.5,"✔","✗"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="18" t="s">
+        <v>147</v>
+      </c>
+      <c r="B25" s="19"/>
+      <c r="C25" s="12" t="str">
+        <f aca="false">IF(B25="","",IF(ABS(B25-Gabarito!$P$14)&lt;0.5,"✔","✗"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="18" t="s">
+        <v>148</v>
+      </c>
+      <c r="B26" s="19"/>
+      <c r="C26" s="12" t="str">
+        <f aca="false">IF(B26="","",IF(ABS(B26-Gabarito!$P$15)&lt;0.5,"✔","✗"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="18" t="s">
+        <v>149</v>
+      </c>
+      <c r="B27" s="19"/>
+      <c r="C27" s="12" t="str">
+        <f aca="false">IF(B27="","",IF(ABS(B27-Gabarito!$P$16)&lt;0.5,"✔","✗"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="18" t="s">
+        <v>99</v>
+      </c>
+      <c r="B28" s="19"/>
+      <c r="C28" s="12" t="str">
+        <f aca="false">IF(B28="","",IF(ABS(B28-Gabarito!$P$17)&lt;0.5,"✔","✗"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="2" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="21"/>
+      <c r="B30" s="21"/>
+      <c r="C30" s="21"/>
+      <c r="D30" s="21"/>
+      <c r="E30" s="21"/>
+      <c r="F30" s="21"/>
+      <c r="G30" s="21"/>
+      <c r="H30" s="21"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A30:H30"/>
+  </mergeCells>
+  <conditionalFormatting sqref="C1:C29">
+    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>"✔"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>"✗"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I1:I18">
+    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>"✔"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="5" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>"✗"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="B1:P36"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="60"/>
@@ -2971,626 +3481,856 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="45"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="0" width="90"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="24"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>119</v>
+        <v>151</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E2" s="9" t="s">
-        <v>120</v>
+        <v>152</v>
       </c>
       <c r="F2" s="9" t="s">
-        <v>121</v>
+        <v>153</v>
       </c>
       <c r="G2" s="9" t="s">
-        <v>122</v>
+        <v>154</v>
       </c>
       <c r="H2" s="9" t="s">
-        <v>123</v>
+        <v>155</v>
+      </c>
+      <c r="J2" s="9" t="s">
+        <v>156</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="4" t="s">
-        <v>124</v>
-      </c>
-      <c r="D3" s="22" t="s">
-        <v>125</v>
-      </c>
-      <c r="E3" s="23" t="n">
+        <v>157</v>
+      </c>
+      <c r="D3" s="26" t="s">
+        <v>158</v>
+      </c>
+      <c r="E3" s="27" t="n">
         <f aca="false">C_Caso1!$C$5</f>
         <v>1000</v>
       </c>
-      <c r="F3" s="23" t="n">
+      <c r="F3" s="27" t="n">
         <f aca="false">C_Caso2!$C$5</f>
         <v>1200</v>
       </c>
+      <c r="I3" s="26" t="s">
+        <v>159</v>
+      </c>
+      <c r="J3" s="27" t="n">
+        <v>50000</v>
+      </c>
+      <c r="K3" s="27" t="n">
+        <v>-30000</v>
+      </c>
+      <c r="L3" s="27" t="n">
+        <v>-6000</v>
+      </c>
+      <c r="M3" s="27" t="n">
+        <v>9000</v>
+      </c>
+      <c r="N3" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" s="27" t="n">
+        <v>-4000</v>
+      </c>
+      <c r="P3" s="27" t="n">
+        <f aca="false">SUM(J3:O3)</f>
+        <v>19000</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D4" s="22" t="s">
-        <v>126</v>
-      </c>
-      <c r="E4" s="23" t="n">
+      <c r="D4" s="26" t="s">
+        <v>160</v>
+      </c>
+      <c r="E4" s="27" t="n">
         <f aca="false">-C_Caso1!$C$6</f>
         <v>-600</v>
       </c>
-      <c r="F4" s="23" t="n">
+      <c r="F4" s="27" t="n">
         <f aca="false">-C_Caso2!$C$6</f>
         <v>-660</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>127</v>
+        <v>161</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>128</v>
+        <v>162</v>
+      </c>
+      <c r="I4" s="26" t="s">
+        <v>163</v>
+      </c>
+      <c r="J4" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" s="27" t="n">
+        <v>8000</v>
+      </c>
+      <c r="O4" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="P4" s="27" t="n">
+        <f aca="false">SUM(J4:O4)</f>
+        <v>8000</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="22" t="s">
-        <v>26</v>
-      </c>
-      <c r="C5" s="22" t="s">
+      <c r="B5" s="26" t="s">
         <v>27</v>
       </c>
-      <c r="D5" s="22" t="s">
-        <v>129</v>
-      </c>
-      <c r="E5" s="23" t="n">
+      <c r="C5" s="26" t="s">
+        <v>28</v>
+      </c>
+      <c r="D5" s="26" t="s">
+        <v>164</v>
+      </c>
+      <c r="E5" s="27" t="n">
         <f aca="false">C_Caso1!$C$5-C_Caso1!$C$6</f>
         <v>400</v>
       </c>
-      <c r="F5" s="23" t="n">
+      <c r="F5" s="27" t="n">
         <f aca="false">C_Caso2!$C$5-C_Caso2!$C$6</f>
         <v>540</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>130</v>
+        <v>165</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>131</v>
+        <v>166</v>
+      </c>
+      <c r="I5" s="26" t="s">
+        <v>167</v>
+      </c>
+      <c r="J5" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" s="27" t="n">
+        <v>12000</v>
+      </c>
+      <c r="M5" s="27" t="n">
+        <v>-6000</v>
+      </c>
+      <c r="N5" s="27" t="n">
+        <v>-4000</v>
+      </c>
+      <c r="O5" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="P5" s="27" t="n">
+        <f aca="false">SUM(J5:O5)</f>
+        <v>2000</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="22" t="s">
+      <c r="B6" s="26" t="s">
+        <v>29</v>
+      </c>
+      <c r="C6" s="26" t="s">
         <v>28</v>
       </c>
-      <c r="C6" s="22" t="s">
-        <v>27</v>
-      </c>
-      <c r="D6" s="22" t="s">
-        <v>132</v>
-      </c>
-      <c r="E6" s="23" t="n">
+      <c r="D6" s="26" t="s">
+        <v>168</v>
+      </c>
+      <c r="E6" s="27" t="n">
         <f aca="false">-C_Caso1!$C$7</f>
         <v>-120</v>
       </c>
-      <c r="F6" s="23" t="n">
+      <c r="F6" s="27" t="n">
         <f aca="false">-C_Caso2!$C$7</f>
         <v>-150</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>133</v>
+        <v>169</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>134</v>
+        <v>170</v>
+      </c>
+      <c r="I6" s="26" t="s">
+        <v>171</v>
+      </c>
+      <c r="J6" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="27" t="n">
+        <v>30000</v>
+      </c>
+      <c r="L6" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="P6" s="27" t="n">
+        <f aca="false">SUM(J6:O6)</f>
+        <v>30000</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="22" t="s">
-        <v>29</v>
-      </c>
-      <c r="C7" s="22" t="s">
-        <v>135</v>
-      </c>
-      <c r="D7" s="22" t="s">
-        <v>136</v>
-      </c>
-      <c r="E7" s="23" t="n">
+      <c r="B7" s="26" t="s">
+        <v>30</v>
+      </c>
+      <c r="C7" s="26" t="s">
+        <v>172</v>
+      </c>
+      <c r="D7" s="26" t="s">
+        <v>173</v>
+      </c>
+      <c r="E7" s="27" t="n">
         <f aca="false">-C_Caso1!$C$8</f>
         <v>-80</v>
       </c>
-      <c r="F7" s="23" t="n">
+      <c r="F7" s="27" t="n">
         <f aca="false">-C_Caso2!$C$8</f>
         <v>-90</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>137</v>
+        <v>174</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>138</v>
+        <v>175</v>
+      </c>
+      <c r="I7" s="26" t="s">
+        <v>176</v>
+      </c>
+      <c r="J7" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" s="27" t="n">
+        <v>6000</v>
+      </c>
+      <c r="M7" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" s="27" t="n">
+        <v>-4000</v>
+      </c>
+      <c r="P7" s="27" t="n">
+        <f aca="false">SUM(J7:O7)</f>
+        <v>2000</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="22" t="s">
-        <v>30</v>
-      </c>
-      <c r="C8" s="22" t="s">
-        <v>139</v>
-      </c>
-      <c r="D8" s="22" t="s">
-        <v>140</v>
-      </c>
-      <c r="E8" s="23" t="n">
+      <c r="B8" s="26" t="s">
+        <v>31</v>
+      </c>
+      <c r="C8" s="26" t="s">
+        <v>177</v>
+      </c>
+      <c r="D8" s="26" t="s">
+        <v>178</v>
+      </c>
+      <c r="E8" s="27" t="n">
         <f aca="false">C_Caso1!$C$5-C_Caso1!$C$6-C_Caso1!$C$7-C_Caso1!$C$8</f>
         <v>200</v>
       </c>
-      <c r="F8" s="23" t="n">
+      <c r="F8" s="27" t="n">
         <f aca="false">C_Caso2!$C$5-C_Caso2!$C$6-C_Caso2!$C$7-C_Caso2!$C$8</f>
         <v>300</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>141</v>
+        <v>179</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>142</v>
+        <v>180</v>
+      </c>
+      <c r="I8" s="26" t="s">
+        <v>181</v>
+      </c>
+      <c r="J8" s="27" t="n">
+        <v>50000</v>
+      </c>
+      <c r="K8" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="P8" s="27" t="n">
+        <f aca="false">SUM(J8:O8)</f>
+        <v>50000</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="C9" s="22" t="s">
-        <v>27</v>
-      </c>
-      <c r="D9" s="22" t="s">
-        <v>143</v>
-      </c>
-      <c r="E9" s="23" t="n">
+      <c r="B9" s="26" t="s">
+        <v>32</v>
+      </c>
+      <c r="C9" s="26" t="s">
+        <v>28</v>
+      </c>
+      <c r="D9" s="26" t="s">
+        <v>182</v>
+      </c>
+      <c r="E9" s="27" t="n">
         <f aca="false">C_Caso1!$C$11-C_Caso1!$C$10</f>
         <v>-30</v>
       </c>
-      <c r="F9" s="23" t="n">
+      <c r="F9" s="27" t="n">
         <f aca="false">C_Caso2!$C$11-C_Caso2!$C$10</f>
         <v>-40</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>144</v>
+        <v>183</v>
+      </c>
+      <c r="I9" s="26" t="s">
+        <v>184</v>
+      </c>
+      <c r="J9" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" s="27" t="n">
+        <v>3000</v>
+      </c>
+      <c r="N9" s="27" t="n">
+        <v>4000</v>
+      </c>
+      <c r="O9" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="P9" s="27" t="n">
+        <f aca="false">SUM(J9:O9)</f>
+        <v>7000</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="22" t="s">
-        <v>32</v>
-      </c>
-      <c r="C10" s="22" t="s">
-        <v>139</v>
-      </c>
-      <c r="D10" s="22" t="s">
-        <v>145</v>
-      </c>
-      <c r="E10" s="23" t="n">
+      <c r="B10" s="26" t="s">
+        <v>33</v>
+      </c>
+      <c r="C10" s="26" t="s">
+        <v>177</v>
+      </c>
+      <c r="D10" s="26" t="s">
+        <v>185</v>
+      </c>
+      <c r="E10" s="27" t="n">
         <f aca="false">C_Caso1!$C$5-C_Caso1!$C$6-C_Caso1!$C$7-C_Caso1!$C$8+C_Caso1!$C$11-C_Caso1!$C$10</f>
         <v>170</v>
       </c>
-      <c r="F10" s="23" t="n">
+      <c r="F10" s="27" t="n">
         <f aca="false">C_Caso2!$C$5-C_Caso2!$C$6-C_Caso2!$C$7-C_Caso2!$C$8+C_Caso2!$C$11-C_Caso2!$C$10</f>
         <v>260</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>146</v>
+        <v>186</v>
+      </c>
+      <c r="I10" s="9" t="s">
+        <v>187</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="22" t="s">
-        <v>33</v>
-      </c>
-      <c r="C11" s="22" t="s">
-        <v>147</v>
-      </c>
-      <c r="D11" s="22" t="s">
-        <v>148</v>
-      </c>
-      <c r="E11" s="23" t="n">
+      <c r="B11" s="26" t="s">
+        <v>34</v>
+      </c>
+      <c r="C11" s="26" t="s">
+        <v>188</v>
+      </c>
+      <c r="D11" s="26" t="s">
+        <v>189</v>
+      </c>
+      <c r="E11" s="27" t="n">
         <f aca="false">-(C_Caso1!$C$5-C_Caso1!$C$6-C_Caso1!$C$7-C_Caso1!$C$8+C_Caso1!$C$11-C_Caso1!$C$10)*C_Caso1!$C$12</f>
         <v>-51</v>
       </c>
-      <c r="F11" s="23" t="n">
+      <c r="F11" s="27" t="n">
         <f aca="false">-(C_Caso2!$C$5-C_Caso2!$C$6-C_Caso2!$C$7-C_Caso2!$C$8+C_Caso2!$C$11-C_Caso2!$C$10)*C_Caso2!$C$12</f>
         <v>-78</v>
       </c>
+      <c r="I11" s="26" t="s">
+        <v>145</v>
+      </c>
+      <c r="P11" s="27" t="n">
+        <v>17000</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="22" t="s">
-        <v>34</v>
-      </c>
-      <c r="C12" s="22" t="s">
-        <v>149</v>
-      </c>
-      <c r="D12" s="22" t="s">
-        <v>150</v>
-      </c>
-      <c r="E12" s="23" t="n">
+      <c r="B12" s="26" t="s">
+        <v>35</v>
+      </c>
+      <c r="C12" s="26" t="s">
+        <v>190</v>
+      </c>
+      <c r="D12" s="26" t="s">
+        <v>191</v>
+      </c>
+      <c r="E12" s="27" t="n">
         <f aca="false">(C_Caso1!$C$5-C_Caso1!$C$6-C_Caso1!$C$7-C_Caso1!$C$8+C_Caso1!$C$11-C_Caso1!$C$10)*(1-C_Caso1!$C$12)</f>
         <v>119</v>
       </c>
-      <c r="F12" s="23" t="n">
+      <c r="F12" s="27" t="n">
         <f aca="false">(C_Caso2!$C$5-C_Caso2!$C$6-C_Caso2!$C$7-C_Caso2!$C$8+C_Caso2!$C$11-C_Caso2!$C$10)*(1-C_Caso2!$C$12)</f>
         <v>182</v>
       </c>
+      <c r="I12" s="26" t="s">
+        <v>78</v>
+      </c>
+      <c r="P12" s="27" t="n">
+        <v>-10000</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D13" s="22" t="s">
-        <v>151</v>
-      </c>
-      <c r="E13" s="24" t="n">
+      <c r="D13" s="26" t="s">
+        <v>192</v>
+      </c>
+      <c r="E13" s="28" t="n">
         <f aca="false">(C_Caso1!$C$5-C_Caso1!$C$6)/C_Caso1!$C$5</f>
         <v>0.4</v>
       </c>
-      <c r="F13" s="24" t="n">
+      <c r="F13" s="28" t="n">
         <f aca="false">(C_Caso2!$C$5-C_Caso2!$C$6)/C_Caso2!$C$5</f>
         <v>0.45</v>
       </c>
+      <c r="I13" s="26" t="s">
+        <v>146</v>
+      </c>
+      <c r="P13" s="27" t="n">
+        <v>7000</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D14" s="22" t="s">
-        <v>152</v>
-      </c>
-      <c r="E14" s="23" t="n">
+      <c r="D14" s="26" t="s">
+        <v>193</v>
+      </c>
+      <c r="E14" s="27" t="n">
         <f aca="false">(C_Caso1!$C$5-C_Caso1!$C$6-C_Caso1!$C$7-C_Caso1!$C$8+C_Caso1!$C$11-C_Caso1!$C$10)*(1-C_Caso1!$C$12)</f>
         <v>119</v>
       </c>
-      <c r="F14" s="23" t="n">
+      <c r="F14" s="27" t="n">
         <f aca="false">(C_Caso2!$C$5-C_Caso2!$C$6-C_Caso2!$C$7-C_Caso2!$C$8+C_Caso2!$C$11-C_Caso2!$C$10)*(1-C_Caso2!$C$12)</f>
         <v>182</v>
       </c>
+      <c r="I14" s="26" t="s">
+        <v>147</v>
+      </c>
+      <c r="P14" s="27" t="n">
+        <v>-1000</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D15" s="22" t="s">
-        <v>153</v>
-      </c>
-      <c r="E15" s="23" t="n">
+      <c r="D15" s="26" t="s">
+        <v>194</v>
+      </c>
+      <c r="E15" s="27" t="n">
         <f aca="false">C_Caso1!$C$9</f>
         <v>30</v>
       </c>
-      <c r="F15" s="23" t="n">
+      <c r="F15" s="27" t="n">
         <f aca="false">C_Caso2!$C$9</f>
         <v>40</v>
       </c>
+      <c r="I15" s="26" t="s">
+        <v>148</v>
+      </c>
+      <c r="P15" s="27" t="n">
+        <v>-30000</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D16" s="22" t="s">
-        <v>154</v>
-      </c>
-      <c r="E16" s="23" t="n">
+      <c r="D16" s="26" t="s">
+        <v>195</v>
+      </c>
+      <c r="E16" s="27" t="n">
         <f aca="false">-C_Caso1!$C$13</f>
         <v>-50</v>
       </c>
-      <c r="F16" s="23" t="n">
+      <c r="F16" s="27" t="n">
         <f aca="false">-C_Caso2!$C$13</f>
         <v>-80</v>
       </c>
+      <c r="I16" s="26" t="s">
+        <v>149</v>
+      </c>
+      <c r="P16" s="27" t="n">
+        <v>50000</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="22" t="s">
-        <v>37</v>
-      </c>
-      <c r="C17" s="22" t="s">
-        <v>155</v>
-      </c>
-      <c r="D17" s="22" t="s">
-        <v>156</v>
-      </c>
-      <c r="E17" s="23" t="n">
+      <c r="B17" s="26" t="s">
+        <v>38</v>
+      </c>
+      <c r="C17" s="26" t="s">
+        <v>196</v>
+      </c>
+      <c r="D17" s="26" t="s">
+        <v>197</v>
+      </c>
+      <c r="E17" s="27" t="n">
         <f aca="false">-C_Caso1!$C$14</f>
         <v>-40</v>
       </c>
-      <c r="F17" s="23" t="n">
+      <c r="F17" s="27" t="n">
         <f aca="false">-C_Caso2!$C$14</f>
         <v>-30</v>
       </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="22" t="s">
-        <v>38</v>
-      </c>
-      <c r="C18" s="22" t="s">
-        <v>157</v>
-      </c>
-      <c r="D18" s="22" t="s">
-        <v>158</v>
-      </c>
-      <c r="E18" s="23" t="n">
+      <c r="I17" s="26" t="s">
+        <v>99</v>
+      </c>
+      <c r="P17" s="27" t="n">
+        <v>19000</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="470.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B18" s="26" t="s">
+        <v>39</v>
+      </c>
+      <c r="C18" s="26" t="s">
+        <v>198</v>
+      </c>
+      <c r="D18" s="26" t="s">
+        <v>199</v>
+      </c>
+      <c r="E18" s="27" t="n">
         <f aca="false">C_Caso1!$C$15</f>
         <v>20</v>
       </c>
-      <c r="F18" s="23" t="n">
+      <c r="F18" s="27" t="n">
         <f aca="false">C_Caso2!$C$15</f>
         <v>50</v>
       </c>
+      <c r="I18" s="26" t="s">
+        <v>200</v>
+      </c>
+      <c r="P18" s="3" t="s">
+        <v>201</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="C19" s="22" t="s">
-        <v>159</v>
-      </c>
-      <c r="D19" s="22" t="s">
-        <v>160</v>
-      </c>
-      <c r="E19" s="23" t="n">
+      <c r="B19" s="26" t="s">
+        <v>40</v>
+      </c>
+      <c r="C19" s="26" t="s">
+        <v>202</v>
+      </c>
+      <c r="D19" s="26" t="s">
+        <v>203</v>
+      </c>
+      <c r="E19" s="27" t="n">
         <f aca="false">((C_Caso1!$C$5-C_Caso1!$C$6-C_Caso1!$C$7-C_Caso1!$C$8+C_Caso1!$C$11-C_Caso1!$C$10)*(1-C_Caso1!$C$12))+C_Caso1!$C$9-C_Caso1!$C$13-C_Caso1!$C$14+C_Caso1!$C$15</f>
         <v>79</v>
       </c>
-      <c r="F19" s="23" t="n">
+      <c r="F19" s="27" t="n">
         <f aca="false">((C_Caso2!$C$5-C_Caso2!$C$6-C_Caso2!$C$7-C_Caso2!$C$8+C_Caso2!$C$11-C_Caso2!$C$10)*(1-C_Caso2!$C$12))+C_Caso2!$C$9-C_Caso2!$C$13-C_Caso2!$C$14+C_Caso2!$C$15</f>
         <v>162</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="C20" s="22" t="s">
-        <v>155</v>
-      </c>
-      <c r="D20" s="22" t="s">
-        <v>160</v>
-      </c>
-      <c r="E20" s="23" t="n">
+      <c r="B20" s="26" t="s">
+        <v>41</v>
+      </c>
+      <c r="C20" s="26" t="s">
+        <v>196</v>
+      </c>
+      <c r="D20" s="26" t="s">
+        <v>203</v>
+      </c>
+      <c r="E20" s="27" t="n">
         <f aca="false">((C_Caso1!$C$5-C_Caso1!$C$6-C_Caso1!$C$7-C_Caso1!$C$8+C_Caso1!$C$11-C_Caso1!$C$10)*(1-C_Caso1!$C$12))+C_Caso1!$C$9-C_Caso1!$C$13-C_Caso1!$C$14+C_Caso1!$C$15</f>
         <v>79</v>
       </c>
-      <c r="F20" s="23" t="n">
+      <c r="F20" s="27" t="n">
         <f aca="false">((C_Caso2!$C$5-C_Caso2!$C$6-C_Caso2!$C$7-C_Caso2!$C$8+C_Caso2!$C$11-C_Caso2!$C$10)*(1-C_Caso2!$C$12))+C_Caso2!$C$9-C_Caso2!$C$13-C_Caso2!$C$14+C_Caso2!$C$15</f>
         <v>162</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="22" t="s">
-        <v>41</v>
-      </c>
-      <c r="C21" s="22" t="s">
-        <v>159</v>
-      </c>
-      <c r="D21" s="22" t="s">
-        <v>161</v>
-      </c>
-      <c r="E21" s="23" t="n">
+      <c r="B21" s="26" t="s">
+        <v>42</v>
+      </c>
+      <c r="C21" s="26" t="s">
+        <v>202</v>
+      </c>
+      <c r="D21" s="26" t="s">
+        <v>204</v>
+      </c>
+      <c r="E21" s="27" t="n">
         <f aca="false">-C_Caso1!$C$16</f>
         <v>-100</v>
       </c>
-      <c r="F21" s="23" t="n">
+      <c r="F21" s="27" t="n">
         <f aca="false">-C_Caso2!$C$16</f>
         <v>-120</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="22" t="s">
-        <v>42</v>
-      </c>
-      <c r="C22" s="22" t="s">
-        <v>155</v>
-      </c>
-      <c r="D22" s="22" t="s">
-        <v>162</v>
-      </c>
-      <c r="E22" s="23" t="n">
+      <c r="B22" s="26" t="s">
+        <v>43</v>
+      </c>
+      <c r="C22" s="26" t="s">
+        <v>196</v>
+      </c>
+      <c r="D22" s="26" t="s">
+        <v>205</v>
+      </c>
+      <c r="E22" s="27" t="n">
         <f aca="false">C_Caso1!$C$17-C_Caso1!$C$18-C_Caso1!$C$19</f>
         <v>30</v>
       </c>
-      <c r="F22" s="23" t="n">
+      <c r="F22" s="27" t="n">
         <f aca="false">C_Caso2!$C$17-C_Caso2!$C$18-C_Caso2!$C$19</f>
         <v>-90</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="22" t="s">
-        <v>43</v>
-      </c>
-      <c r="C23" s="22" t="s">
-        <v>157</v>
-      </c>
-      <c r="D23" s="22" t="s">
-        <v>163</v>
-      </c>
-      <c r="E23" s="23" t="n">
+      <c r="B23" s="26" t="s">
+        <v>44</v>
+      </c>
+      <c r="C23" s="26" t="s">
+        <v>198</v>
+      </c>
+      <c r="D23" s="26" t="s">
+        <v>206</v>
+      </c>
+      <c r="E23" s="27" t="n">
         <f aca="false">(((C_Caso1!$C$5-C_Caso1!$C$6-C_Caso1!$C$7-C_Caso1!$C$8+C_Caso1!$C$11-C_Caso1!$C$10)*(1-C_Caso1!$C$12))+C_Caso1!$C$9-C_Caso1!$C$13-C_Caso1!$C$14+C_Caso1!$C$15)+(-C_Caso1!$C$16)+(C_Caso1!$C$17-C_Caso1!$C$18-C_Caso1!$C$19)</f>
         <v>9</v>
       </c>
-      <c r="F23" s="23" t="n">
+      <c r="F23" s="27" t="n">
         <f aca="false">(((C_Caso2!$C$5-C_Caso2!$C$6-C_Caso2!$C$7-C_Caso2!$C$8+C_Caso2!$C$11-C_Caso2!$C$10)*(1-C_Caso2!$C$12))+C_Caso2!$C$9-C_Caso2!$C$13-C_Caso2!$C$14+C_Caso2!$C$15)+(-C_Caso2!$C$16)+(C_Caso2!$C$17-C_Caso2!$C$18-C_Caso2!$C$19)</f>
         <v>-48</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="22" t="s">
-        <v>44</v>
-      </c>
-      <c r="C24" s="22" t="s">
-        <v>155</v>
-      </c>
-      <c r="D24" s="22" t="s">
-        <v>164</v>
-      </c>
-      <c r="E24" s="23" t="n">
+      <c r="B24" s="26" t="s">
+        <v>45</v>
+      </c>
+      <c r="C24" s="26" t="s">
+        <v>196</v>
+      </c>
+      <c r="D24" s="26" t="s">
+        <v>207</v>
+      </c>
+      <c r="E24" s="27" t="n">
         <f aca="false">((((C_Caso1!$C$5-C_Caso1!$C$6-C_Caso1!$C$7-C_Caso1!$C$8+C_Caso1!$C$11-C_Caso1!$C$10)*(1-C_Caso1!$C$12))+C_Caso1!$C$9-C_Caso1!$C$13-C_Caso1!$C$14+C_Caso1!$C$15)+(-C_Caso1!$C$16)+(C_Caso1!$C$17-C_Caso1!$C$18-C_Caso1!$C$19))+C_Caso1!$C$20</f>
         <v>50</v>
       </c>
-      <c r="F24" s="23" t="n">
+      <c r="F24" s="27" t="n">
         <f aca="false">((((C_Caso2!$C$5-C_Caso2!$C$6-C_Caso2!$C$7-C_Caso2!$C$8+C_Caso2!$C$11-C_Caso2!$C$10)*(1-C_Caso2!$C$12))+C_Caso2!$C$9-C_Caso2!$C$13-C_Caso2!$C$14+C_Caso2!$C$15)+(-C_Caso2!$C$16)+(C_Caso2!$C$17-C_Caso2!$C$18-C_Caso2!$C$19))+C_Caso2!$C$20</f>
         <v>52</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D25" s="22" t="s">
-        <v>165</v>
-      </c>
-      <c r="E25" s="23" t="n">
+      <c r="D25" s="26" t="s">
+        <v>208</v>
+      </c>
+      <c r="E25" s="27" t="n">
         <f aca="false">(((C_Caso1!$C$5-C_Caso1!$C$6-C_Caso1!$C$7-C_Caso1!$C$8+C_Caso1!$C$11-C_Caso1!$C$10)*(1-C_Caso1!$C$12))+C_Caso1!$C$9-C_Caso1!$C$13-C_Caso1!$C$14+C_Caso1!$C$15)+(-C_Caso1!$C$16)+(C_Caso1!$C$17-C_Caso1!$C$18-C_Caso1!$C$19)</f>
         <v>9</v>
       </c>
-      <c r="F25" s="23" t="n">
+      <c r="F25" s="27" t="n">
         <f aca="false">(((C_Caso2!$C$5-C_Caso2!$C$6-C_Caso2!$C$7-C_Caso2!$C$8+C_Caso2!$C$11-C_Caso2!$C$10)*(1-C_Caso2!$C$12))+C_Caso2!$C$9-C_Caso2!$C$13-C_Caso2!$C$14+C_Caso2!$C$15)+(-C_Caso2!$C$16)+(C_Caso2!$C$17-C_Caso2!$C$18-C_Caso2!$C$19)</f>
         <v>-48</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D26" s="22" t="s">
-        <v>166</v>
-      </c>
-      <c r="E26" s="23" t="n">
+      <c r="D26" s="26" t="s">
+        <v>209</v>
+      </c>
+      <c r="E26" s="27" t="n">
         <f aca="false">C_Caso1!$C$13</f>
         <v>50</v>
       </c>
-      <c r="F26" s="23" t="n">
+      <c r="F26" s="27" t="n">
         <f aca="false">C_Caso2!$C$13</f>
         <v>80</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D27" s="22" t="s">
-        <v>167</v>
-      </c>
-      <c r="E27" s="23" t="n">
+      <c r="D27" s="26" t="s">
+        <v>210</v>
+      </c>
+      <c r="E27" s="27" t="n">
         <f aca="false">C_Caso1!$C$14</f>
         <v>40</v>
       </c>
-      <c r="F27" s="23" t="n">
+      <c r="F27" s="27" t="n">
         <f aca="false">C_Caso2!$C$14</f>
         <v>30</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D28" s="22" t="s">
-        <v>168</v>
-      </c>
-      <c r="E28" s="23" t="n">
+      <c r="D28" s="26" t="s">
+        <v>211</v>
+      </c>
+      <c r="E28" s="27" t="n">
         <f aca="false">C_Caso1!$C$16-C_Caso1!$C$9</f>
         <v>70</v>
       </c>
-      <c r="F28" s="23" t="n">
+      <c r="F28" s="27" t="n">
         <f aca="false">C_Caso2!$C$16-C_Caso2!$C$9</f>
         <v>80</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B29" s="22" t="s">
-        <v>46</v>
-      </c>
-      <c r="C29" s="22" t="s">
-        <v>169</v>
-      </c>
-      <c r="D29" s="22" t="s">
-        <v>170</v>
-      </c>
-      <c r="E29" s="23" t="n">
+      <c r="B29" s="26" t="s">
+        <v>47</v>
+      </c>
+      <c r="C29" s="26" t="s">
+        <v>148</v>
+      </c>
+      <c r="D29" s="26" t="s">
+        <v>212</v>
+      </c>
+      <c r="E29" s="27" t="n">
         <f aca="false">((((C_Caso1!$C$5-C_Caso1!$C$6-C_Caso1!$C$7-C_Caso1!$C$8+C_Caso1!$C$11-C_Caso1!$C$10)*(1-C_Caso1!$C$12))+C_Caso1!$C$9-C_Caso1!$C$13-C_Caso1!$C$14+C_Caso1!$C$15)+(-C_Caso1!$C$16)+(C_Caso1!$C$17-C_Caso1!$C$18-C_Caso1!$C$19))+C_Caso1!$C$13+C_Caso1!$C$14+C_Caso1!$C$16-C_Caso1!$C$9</f>
         <v>169</v>
       </c>
-      <c r="F29" s="23" t="n">
+      <c r="F29" s="27" t="n">
         <f aca="false">((((C_Caso2!$C$5-C_Caso2!$C$6-C_Caso2!$C$7-C_Caso2!$C$8+C_Caso2!$C$11-C_Caso2!$C$10)*(1-C_Caso2!$C$12))+C_Caso2!$C$9-C_Caso2!$C$13-C_Caso2!$C$14+C_Caso2!$C$15)+(-C_Caso2!$C$16)+(C_Caso2!$C$17-C_Caso2!$C$18-C_Caso2!$C$19))+C_Caso2!$C$13+C_Caso2!$C$14+C_Caso2!$C$16-C_Caso2!$C$9</f>
         <v>142</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B30" s="22" t="s">
-        <v>47</v>
-      </c>
-      <c r="C30" s="22" t="s">
-        <v>171</v>
-      </c>
-      <c r="D30" s="22" t="s">
-        <v>172</v>
-      </c>
-      <c r="E30" s="23" t="n">
+      <c r="B30" s="26" t="s">
+        <v>48</v>
+      </c>
+      <c r="C30" s="26" t="s">
+        <v>213</v>
+      </c>
+      <c r="D30" s="26" t="s">
+        <v>214</v>
+      </c>
+      <c r="E30" s="27" t="n">
         <f aca="false">C_Caso1!$C$15</f>
         <v>20</v>
       </c>
-      <c r="F30" s="23" t="n">
+      <c r="F30" s="27" t="n">
         <f aca="false">C_Caso2!$C$15</f>
         <v>50</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B31" s="22" t="s">
-        <v>48</v>
-      </c>
-      <c r="C31" s="22" t="s">
-        <v>173</v>
-      </c>
-      <c r="D31" s="22" t="s">
-        <v>174</v>
-      </c>
-      <c r="E31" s="23" t="n">
+      <c r="B31" s="26" t="s">
+        <v>49</v>
+      </c>
+      <c r="C31" s="26" t="s">
+        <v>149</v>
+      </c>
+      <c r="D31" s="26" t="s">
+        <v>215</v>
+      </c>
+      <c r="E31" s="27" t="n">
         <f aca="false">C_Caso1!$C$17-C_Caso1!$C$18</f>
         <v>60</v>
       </c>
-      <c r="F31" s="23" t="n">
+      <c r="F31" s="27" t="n">
         <f aca="false">C_Caso2!$C$17-C_Caso2!$C$18</f>
         <v>-40</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B32" s="22" t="s">
-        <v>49</v>
-      </c>
-      <c r="C32" s="22" t="s">
-        <v>173</v>
-      </c>
-      <c r="D32" s="22" t="s">
-        <v>175</v>
-      </c>
-      <c r="E32" s="23" t="n">
+      <c r="B32" s="26" t="s">
+        <v>50</v>
+      </c>
+      <c r="C32" s="26" t="s">
+        <v>149</v>
+      </c>
+      <c r="D32" s="26" t="s">
+        <v>216</v>
+      </c>
+      <c r="E32" s="27" t="n">
         <f aca="false">((C_Caso1!$C$5-C_Caso1!$C$6-C_Caso1!$C$7-C_Caso1!$C$8+C_Caso1!$C$11-C_Caso1!$C$10)*(1-C_Caso1!$C$12))-C_Caso1!$C$19</f>
         <v>89</v>
       </c>
-      <c r="F32" s="23" t="n">
+      <c r="F32" s="27" t="n">
         <f aca="false">((C_Caso2!$C$5-C_Caso2!$C$6-C_Caso2!$C$7-C_Caso2!$C$8+C_Caso2!$C$11-C_Caso2!$C$10)*(1-C_Caso2!$C$12))-C_Caso2!$C$19</f>
         <v>132</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B33" s="22" t="s">
-        <v>50</v>
-      </c>
-      <c r="C33" s="22" t="s">
-        <v>169</v>
-      </c>
-      <c r="D33" s="22" t="s">
-        <v>176</v>
-      </c>
-      <c r="E33" s="23" t="n">
+      <c r="B33" s="26" t="s">
+        <v>51</v>
+      </c>
+      <c r="C33" s="26" t="s">
+        <v>148</v>
+      </c>
+      <c r="D33" s="26" t="s">
+        <v>217</v>
+      </c>
+      <c r="E33" s="27" t="n">
         <f aca="false">C_Caso1!$C$15+C_Caso1!$C$17-C_Caso1!$C$18+((C_Caso1!$C$5-C_Caso1!$C$6-C_Caso1!$C$7-C_Caso1!$C$8+C_Caso1!$C$11-C_Caso1!$C$10)*(1-C_Caso1!$C$12))-C_Caso1!$C$19</f>
         <v>169</v>
       </c>
-      <c r="F33" s="23" t="n">
+      <c r="F33" s="27" t="n">
         <f aca="false">C_Caso2!$C$15+C_Caso2!$C$17-C_Caso2!$C$18+((C_Caso2!$C$5-C_Caso2!$C$6-C_Caso2!$C$7-C_Caso2!$C$8+C_Caso2!$C$11-C_Caso2!$C$10)*(1-C_Caso2!$C$12))-C_Caso2!$C$19</f>
         <v>142</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="255.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B34" s="22" t="s">
-        <v>51</v>
-      </c>
-      <c r="C34" s="22" t="s">
-        <v>171</v>
-      </c>
-      <c r="D34" s="22" t="s">
-        <v>177</v>
+      <c r="B34" s="26" t="s">
+        <v>52</v>
+      </c>
+      <c r="C34" s="26" t="s">
+        <v>213</v>
+      </c>
+      <c r="D34" s="26" t="s">
+        <v>218</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>178</v>
+        <v>219</v>
       </c>
       <c r="F34" s="3" t="s">
-        <v>179</v>
+        <v>220</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B35" s="22" t="s">
-        <v>52</v>
-      </c>
-      <c r="C35" s="22" t="s">
-        <v>173</v>
+      <c r="B35" s="26" t="s">
+        <v>53</v>
+      </c>
+      <c r="C35" s="26" t="s">
+        <v>149</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B36" s="22" t="s">
-        <v>53</v>
-      </c>
-      <c r="C36" s="22" t="s">
-        <v>169</v>
+      <c r="B36" s="26" t="s">
+        <v>54</v>
+      </c>
+      <c r="C36" s="26" t="s">
+        <v>148</v>
       </c>
     </row>
   </sheetData>

</xml_diff>